<commit_message>
docs(domain-model): review the identity tables
Design review of 2026-10-04, tables 1-11 (organizations to
access_audit_logs), nothing implemented yet: status_reason on decided
statuses (DM-19), memberships tracked in change history (DM-20), login
lockout and activity in user_state, user_devices became user_sessions,
one-time codes, three-level legal acceptance with legal_documents,
exactly one ORG_ADMIN per organization enforced by a unique index, a
two-column foreign key keeping role assignments in their membership's
organization, and security events plus a details column in
access_audit_logs. Decisions ID-22 to ID-42 recorded; feature catalog
updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -4418,7 +4418,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="40.5" customHeight="1">
+    <row r="16" ht="54" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>PAY-12</t>
@@ -4447,7 +4447,7 @@
       <c r="F16" s="3" t="inlineStr">
         <is>
           <t>• Chiến dịch với đối tượng, thời gian và ưu đãi
-• Chỉ gửi khi có đồng ý nhận tin tiếp thị
+• Chỉ gửi khi có đồng ý nhận tin tiếp thị (cơ chế đồng ý/từ chối được thiết kế cùng tính năng này)
 • Áp dụng giảm giá cho sạc hoặc dịch vụ</t>
         </is>
       </c>
@@ -10376,7 +10376,7 @@
       <c r="F7" s="3" t="inlineStr">
         <is>
           <t>• Hồ sơ: họ tên, số điện thoại (tên đăng nhập), e-mail không bắt buộc
-• Trạng thái Đã mời / Hoạt động / Bị khóa; chỉ quản trị nội bộ được khóa cả tài khoản
+• Trạng thái Đã mời / Hoạt động / Bị khóa, kèm lý do; chỉ quản trị nội bộ được khóa cả tài khoản
 • Ghi nhận ai tạo tài khoản và lưu lịch sử thay đổi</t>
         </is>
       </c>
@@ -10424,7 +10424,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="108" customHeight="1">
+    <row r="8" ht="216" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>ACC-04</t>
@@ -10453,10 +10453,12 @@
       <c r="F8" s="3" t="inlineStr">
         <is>
           <t>• Đăng nhập bằng SĐT + mật khẩu, đăng xuất, hết hạn phiên
+• Xem các thiết bị đang đăng nhập và đăng xuất từng thiết bị hoặc tất cả; mọi phiên kết thúc khi đổi mật khẩu hoặc tài khoản bị khóa
 • Chọn tổ chức sau khi đăng nhập, nhớ tổ chức dùng gần nhất
-• Tạm khóa sau nhiều lần đăng nhập sai
+• Tạm khóa sau nhiều lần đăng nhập sai, kèm giới hạn số lần thử theo thiết bị/IP; vẫn đặt lại mật khẩu bằng OTP được trong lúc bị khóa
 • Mật khẩu chỉ lưu dạng băm một chiều; không dùng lại mật khẩu cũ
-• Ghi nhận lần đăng nhập và hoạt động gần nhất</t>
+• Ghi nhận lần đăng nhập và hoạt động gần nhất
+• Lịch sử đăng nhập (thời gian, IP, thiết bị) cho người dùng và quản trị nội bộ xem; báo người dùng khi đăng nhập từ thiết bị mới</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -10503,7 +10505,7 @@
       </c>
       <c r="Q8" s="3" t="n"/>
     </row>
-    <row r="9" ht="67.5" customHeight="1">
+    <row r="9" ht="94.5" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ACC-05</t>
@@ -10531,7 +10533,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>• Mã được băm, có hạn dùng và chỉ dùng một lần
+          <t>• Mã được băm, có hạn dùng và chỉ dùng một lần; nhập sai 5 lần thì mã hết hiệu lực; chỉ mã mới nhất được tính
 • Giới hạn số lần gửi theo SĐT để chống lạm dụng và tiết kiệm chi phí SMS
 • Một cơ chế dùng chung cho đăng ký, lời mời, đặt lại mật khẩu và đổi SĐT</t>
         </is>
@@ -10580,7 +10582,7 @@
       </c>
       <c r="Q9" s="3" t="n"/>
     </row>
-    <row r="10" ht="67.5" customHeight="1">
+    <row r="10" ht="108" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>ACC-06</t>
@@ -10610,7 +10612,8 @@
         <is>
           <t>• Quên mật khẩu: OTP gửi tới SĐT đã đăng ký, rồi đặt mật khẩu mới
 • Đổi SĐT: OTP gửi tới số mới; thay đổi được lưu lịch sử
-• Đổi mật khẩu khi đang đăng nhập</t>
+• Đổi mật khẩu khi đang đăng nhập
+• CSKH hoặc quản trị tổ chức xác minh thêm trước khi đặt lại mật khẩu cho tài khoản lâu không hoạt động (số điện thoại có thể bị nhà mạng cấp lại)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -10735,7 +10738,7 @@
       </c>
       <c r="Q11" s="3" t="n"/>
     </row>
-    <row r="12" ht="40.5" customHeight="1">
+    <row r="12" ht="67.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>ACC-08</t>
@@ -10765,7 +10768,8 @@
         <is>
           <t>• Tạo tổ chức và gói thuê bao trong một luồng
 • Mời quản trị viên đầu tiên của tổ chức qua SĐT
-• Gán nhân viên phụ trách</t>
+• Gán nhân viên phụ trách
+• Quản trị viên đầu tiên chấp thuận thỏa thuận xử lý dữ liệu thay mặt doanh nghiệp ở lần đăng nhập đầu</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -11041,7 +11045,7 @@
       </c>
       <c r="Q15" s="3" t="n"/>
     </row>
-    <row r="16" ht="54" customHeight="1">
+    <row r="16" ht="67.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>ACC-12</t>
@@ -11070,7 +11074,7 @@
       <c r="F16" s="3" t="inlineStr">
         <is>
           <t>• Danh sách thành viên của tổ chức kèm vai trò
-• Khóa, mở khóa hoặc cho thành viên rời tổ chức (vẫn giữ lịch sử)
+• Khóa, mở khóa hoặc cho thành viên rời tổ chức kèm lý do (vẫn giữ lịch sử); xem thời điểm mời và thời điểm tham gia của từng thành viên
 • Người dùng xem và chuyển giữa các tổ chức của mình</t>
         </is>
       </c>
@@ -11118,7 +11122,7 @@
       </c>
       <c r="Q16" s="3" t="n"/>
     </row>
-    <row r="17" ht="81" customHeight="1">
+    <row r="17" ht="108" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>ACC-13</t>
@@ -11146,8 +11150,8 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>• Gán và thu hồi vai trò theo từng thành viên, có lịch sử
-• Luôn còn ít nhất một quản trị tổ chức đang hoạt động
+          <t>• Gán và thu hồi vai trò theo từng thành viên, có lịch sử: ai đã cấp hoặc thu hồi từng vai trò, và khi nào
+• Đúng một quản trị tổ chức: chuyển giao vai trò trong một bước; đồng quản trị của chúng ta chỉ định người mới khi quản trị viên không còn
 • Vai trò quản trị trưởng và đồng quản trị chỉ có ở tổ chức nội bộ; đồng quản trị không quản lý được quản trị viên</t>
         </is>
       </c>
@@ -11358,7 +11362,7 @@
       </c>
       <c r="Q19" s="3" t="n"/>
     </row>
-    <row r="20" ht="54" customHeight="1">
+    <row r="20" ht="94.5" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>ACC-16</t>
@@ -11386,8 +11390,9 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>• Lưu token Firebase theo thiết bị, làm mới khi đăng nhập
-• Xóa token khi đăng xuất, khi bị báo hủy đăng ký và khi quá cũ</t>
+          <t>• Lưu token Firebase trên phiên đăng nhập của thiết bị, làm mới khi đăng nhập; không bắt buộc khi người dùng từ chối thông báo
+• Token mất cùng với phiên: đăng xuất, hết hạn, đổi mật khẩu, khóa tài khoản, hoặc app bị báo đã gỡ
+• Thông báo của mọi tổ chức của người dùng tới mọi thiết bị; mở thông báo sẽ chuyển sang tổ chức của nó</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -11434,7 +11439,7 @@
       </c>
       <c r="Q20" s="3" t="n"/>
     </row>
-    <row r="21" ht="67.5" customHeight="1">
+    <row r="21" ht="189" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ACC-17</t>
@@ -11442,30 +11447,31 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Quản lý đồng ý xử lý dữ liệu</t>
+          <t>Chấp thuận văn bản pháp lý &amp; đồng ý xử lý dữ liệu</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Ghi nhận việc mỗi người đồng ý điều khoản, chính sách quyền riêng tư và theo dõi vị trí, theo từng phiên bản văn bản, và cho phép rút lại.</t>
+          <t>Ghi nhận ai đã chấp thuận phiên bản nào của văn bản pháp lý nào: doanh nghiệp chấp thuận thỏa thuận xử lý dữ liệu thay mặt chính mình, tài xế là nhân viên xác nhận đã đọc thông báo quyền riêng tư, khách hàng cá nhân chấp thuận điều khoản, chính sách quyền riêng tư và theo dõi vị trí.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Chứng minh việc xử lý dữ liệu cá nhân đúng luật (Nghị định 13/2023, Luật 91/2025/QH15).</t>
+          <t>Chứng minh việc xử lý dữ liệu cá nhân đúng luật (Nghị định 13/2023, Luật 91/2025/QH15) bằng đúng văn bản đã được chấp thuận.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Tài xế, Quản trị tổ chức, Hệ thống (tự động)</t>
+          <t>Tài xế, Quản trị tổ chức, Đồng quản trị (nội bộ), Hệ thống (tự động)</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>• Xin đồng ý khi kích hoạt, theo từng mục đích, kèm phiên bản văn bản
-• Rút lại đồng ý; ghi nhận thời điểm và kênh
-• Xin đồng ý lại khi văn bản thay đổi
-• Chỉ gửi tin tiếp thị khi có đồng ý nhận tin tiếp thị</t>
+          <t>• Công bố các phiên bản của từng văn bản pháp lý; phiên bản mới yêu cầu mọi người liên quan chấp thuận lại trước khi tiếp tục
+• Quản trị tổ chức chấp thuận thỏa thuận xử lý dữ liệu thay mặt doanh nghiệp ở lần đăng nhập đầu; thành viên chưa dùng được hệ thống trước đó
+• Tài xế là nhân viên xác nhận đã đọc thông báo quyền riêng tư mỗi phiên bản một lần; khách hàng cá nhân đồng ý theo từng mục đích
+• Bằng chứng lưu kèm mỗi lần chấp thuận: đúng phiên bản văn bản, thời điểm, IP và thiết bị; không bao giờ sửa
+• Rút lại chấp thuận bắt buộc nghĩa là ngừng sử dụng dịch vụ (đóng tài khoản)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -11502,17 +11508,17 @@
       <c r="N21" s="3" t="n"/>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>• Khi tài xế rút đồng ý theo dõi vị trí, xe của doanh nghiệp có còn được theo dõi vị trí không?</t>
+          <t>• Luật sư cần xác nhận mô hình thỏa thuận với doanh nghiệp tại Việt Nam (câu hỏi mở 6).</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-37, NF-08, Quyết định ID-20</t>
+          <t>Bảng dữ liệu IN-37, NF-08, Quyết định ID-20, Quyết định ID-38</t>
         </is>
       </c>
       <c r="Q21" s="3" t="n"/>
     </row>
-    <row r="22" ht="81" customHeight="1">
+    <row r="22" ht="148.5" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>ACC-18</t>
@@ -11542,7 +11548,9 @@
         <is>
           <t>• Nhật ký chỉ ghi thêm cho mọi lần truy cập dữ liệu cá nhân, vị trí và camera
 • Yêu cầu lý do hoặc mã ticket trước khi trích xuất dữ liệu nhạy cảm
-• Tra cứu nhật ký theo người truy cập, người được truy cập, thời gian và loại dữ liệu</t>
+• Tra cứu nhật ký theo người truy cập, tổ chức, thời gian và loại dữ liệu
+• Ghi một dòng mỗi lần mở màn hình (không ghi mỗi lần làm mới); lưu vĩnh viễn, các tháng cũ được nén
+• Sự kiện bảo mật tài khoản trong cùng nhật ký: đăng nhập, đăng nhập sai, bị khóa tạm, đăng xuất, đổi mật khẩu và số điện thoại, kèm IP và thiết bị</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): review the vehicles table
Design review of 2026-10-04, table 12, nothing implemented yet. The
vehicle status is a service status set by a person (ACTIVE, MAINTENANCE,
DECOMMISSIONED) with a reason; INACTIVE is dropped since idleness is
computed (VH-05). activation_status is dropped and vehicles gets no state
table: everything the truck reports is kept in vehicle_telemetry (VH-06,
supersedes VH-01). Vehicles keep change history; VIN and plate are
editable and unique among live trucks; organization_id is the current
owner (VH-07). Batteries become managed assets and warranties get their
own table, both to be designed after table 13 (VH-08, VH-09); pack/cell
management and battery leasing deferred (items 87, 88). A truck may have
several drivers at once (DR-05). Feature catalog updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -12700,7 +12700,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40.5" customHeight="1">
+    <row r="5" ht="135" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>VEH-01</t>
@@ -12713,7 +12713,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Lưu hồ sơ từng xe: số VIN, biển số, dòng xe, ngày bàn giao, trạng thái bảo hành và trạng thái hoạt động.</t>
+          <t>Lưu hồ sơ từng xe: số VIN, biển số, dòng xe, ngày bàn giao, trạng thái bảo hành và trạng thái phục vụ.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -12729,7 +12729,9 @@
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>• Tạo, sửa, tìm kiếm và ngừng sử dụng xe
-• VIN và biển số không trùng; lưu lịch sử thay đổi
+• VIN và biển số không trùng trong các xe đang dùng và đều sửa được (nhập nhầm, biển số theo chủ xe); lưu lịch sử thay đổi kèm lý do
+• Trạng thái phục vụ do con người đặt: đang phục vụ, đang bảo dưỡng, đã rời hệ thống, kèm lý do; xe nhàn rỗi hay mất tín hiệu được hiển thị từ dữ liệu, không lưu
+• Bảo hành theo từng xe, pin và thiết bị với giới hạn riêng; bảo hành bị hủy lưu kèm lý do
 • Lọc theo trạng thái, dòng xe, chủ sở hữu và đội xe</t>
         </is>
       </c>
@@ -12765,14 +12767,10 @@
       </c>
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>• Biển số có được thay đổi sau khi đăng ký không (đăng ký lại, sang tên)?</t>
-        </is>
-      </c>
+      <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, PRD F-F2</t>
+          <t>Bảng dữ liệu IN-32, PRD F-F2, Quyết định VH-05, Quyết định VH-07, Quyết định VH-09</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -12932,12 +12930,12 @@
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, Bảng dữ liệu IN-34, deferred.md 61</t>
+          <t>Bảng dữ liệu IN-32, Bảng dữ liệu IN-34, deferred.md 61, Quyết định VH-08</t>
         </is>
       </c>
       <c r="Q7" s="3" t="n"/>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="67.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>VEH-04</t>
@@ -12950,12 +12948,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Lưu hồ sơ từng pack pin: hóa học pin, dung lượng thiết kế và sơ đồ cell/module (mã cell và vị trí).</t>
+          <t>Quản lý từng pin xe như một tài sản: dòng pin, chủ sở hữu và các xe pin đã được lắp.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cho phép chẩn đoán cấp cell và thay cell đơn lẻ.</t>
+          <t>Pin chiếm tới hai phần ba giá xe; sức khỏe, bảo hành và giá trị của pin đi theo pin từ xe này sang xe khác.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -12965,9 +12963,9 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>• Mã pack, hóa học (LFP/CATL), dung lượng thiết kế, gắn với xe
-• Sơ đồ cell/module: số lượng, mã và vị trí
-• Lịch sử thay pack</t>
+          <t>• Danh mục dòng pin: hóa học (LFP/CATL), dung lượng thiết kế, điện áp, cấu trúc
+• Từng pin: số serial, dòng pin, chủ sở hữu (có thể khác chủ xe), trạng thái kèm lý do
+• Mỗi xe một pin; lịch sử pin đã được lắp trên xe nào</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -13009,7 +13007,7 @@
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-33</t>
+          <t>Bảng dữ liệu IN-33, Quyết định VH-08, deferred.md 87, deferred.md 88</t>
         </is>
       </c>
       <c r="Q8" s="3" t="n"/>
@@ -13042,7 +13040,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>• Các bước kích hoạt: chờ, đã gắn thiết bị, đã kích hoạt khi có dữ liệu đầu tiên
+          <t>• Kích hoạt được tính từ thiết bị đang lắp và dữ liệu đã nhận, nên xe bị tháo T-Box sẽ hiện đúng như vậy
 • Tỷ lệ kích hoạt thành công và danh sách xe còn đang chờ</t>
         </is>
       </c>
@@ -13085,7 +13083,7 @@
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>PRD F-F2, Quyết định VH-01</t>
+          <t>PRD F-F2, Quyết định VH-06</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -16569,7 +16567,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>• Mỗi tài xế một xe và mỗi xe một tài xế đang hoạt động
+          <t>• Mỗi tài xế một xe đang hoạt động; một xe có thể có nhiều tài xế cùng lúc (chia ca, lái phụ)
 • Đổi xe trong một bước; lịch sử theo tài xế và theo xe</t>
         </is>
       </c>
@@ -16616,7 +16614,7 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-01</t>
+          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-01, Quyết định DR-05</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): replace driver assignments with driver check-in
Design review of 2026-10-04, nothing implemented yet. A driving_sessions
table records who is at the wheel: the driver scans the truck's QR code,
picks a nearby truck in the app, or is checked in from the portal. Any
active driver may check in to any organization's truck, with a warning
when the driver is from another organization; a session ends at
check-out, takeover, another truck or the organization's auto-end time
(DR-07, supersedes DR-01, DR-05, DR-06). driver_vehicle_assignments will
be dropped. Organization settings get their own table (ID-45); driver
alerts go to the driver checked in and the portal (NT-07); two planned
notification types. DRV-02 becomes "Driver check-in".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -917,7 +917,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>0/5</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>0/63</t>
+          <t>0/64</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
@@ -16539,7 +16539,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="189" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>DRV-02</t>
@@ -16547,28 +16547,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Phân công xe</t>
+          <t>Nhận xe</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Giao và đổi xe cho tài xế, lưu toàn bộ lịch sử phân công.</t>
+          <t>Tài xế nhận chiếc xe sắp lái bằng cách quét mã QR trên xe hoặc chọn xe trên ứng dụng; hệ thống luôn biết ai đang cầm lái và lưu toàn bộ lịch sử.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Mọi sự kiện của xe đều truy được tài xế tại thời điểm đó.</t>
+          <t>Trong vận tải chặng ngắn, tài xế và xe đổi nhau hằng ngày; mọi sự kiện của xe vẫn truy được tài xế tại thời điểm đó.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Quản lý đội xe, Điều vận</t>
+          <t>Tài xế, Quản lý đội xe, Điều vận, Hệ thống (tự động)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>• Mỗi tài xế một xe đang hoạt động; một xe có thể có nhiều tài xế cùng lúc (chia ca, lái phụ)
-• Đổi xe trong một bước; lịch sử theo tài xế và theo xe</t>
+          <t>• Nhận xe bằng cách quét mã QR trên xe hoặc chọn xe ở gần trên ứng dụng, bị từ chối khi điện thoại ở xa xe; quản lý có thể nhận xe giúp tài xế trên portal
+• Tài xế đang hoạt động nào cũng có thể lái xe của bất kỳ tổ chức nào; cảnh báo khi tài xế thuộc tổ chức khác
+• Mỗi xe một người cầm lái; phiên kết thúc khi trả xe, khi tài xế khác nhận xe, khi tài xế nhận xe khác, hoặc khi xe không di chuyển quá thời gian tự kết thúc của tổ chức (mặc định 2 giờ)
+• Cảnh báo lên portal khi xe chạy mà không ai nhận xe
+• Cảnh báo dành cho tài xế gửi tới tài xế đang nhận xe và portal
+• Lịch sử theo tài xế và theo xe</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -16593,7 +16597,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Không cần</t>
+          <t>Chưa làm</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -16607,14 +16611,10 @@
         </is>
       </c>
       <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>• Hai tài xế dùng chung một xe theo ca: một hay hai tài khoản app? (xem DRV-04)</t>
-        </is>
-      </c>
+      <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-01, Quyết định DR-05</t>
+          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-07, Quyết định NT-07, Quyết định ID-45</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): keep vehicle ownership on the vehicle and answer D3
A relationship where A belongs to at most one B at a time is a column plus
a since column with change history, its periods read from the history
through a view (DM-22). Vehicle ownership follows it: owned_since on
vehicles, the proposed vehicle_ownerships table dropped (VH-10). After a
sale, the previous owner keeps the rows recorded under it, while the
truck's condition and lifetime totals follow the truck (VH-11, answers
D3). One transfer action closes the seller's fleet memberships, driving
session, charging rules, subscription and VIN credential (VH-12).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -12779,7 +12779,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40.5" customHeight="1">
+    <row r="6" ht="108" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>VEH-02</t>
@@ -12808,7 +12808,8 @@
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>• Ghi nhận chủ sở hữu khi bàn giao
-• Chuyển quyền sở hữu kèm ngày hiệu lực; lưu lịch sử</t>
+• Chuyển quyền sở hữu kèm ngày hiệu lực trong một bước: tư cách thành viên đội xe, phiên lái, quy tắc sạc, thuê bao và thẻ sạc theo VIN của bên bán đối với xe kết thúc cùng lúc
+• Chủ cũ giữ dữ liệu của mình trước ngày bán; tình trạng xe và các tổng tích lũy đi theo xe sang chủ mới; mọi giai đoạn sở hữu kèm người ghi nhận và lý do</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -12847,14 +12848,10 @@
         </is>
       </c>
       <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>• Sau khi đổi chủ, chủ mới có xem được dữ liệu của xe trước ngày chuyển không? (quyết định mở D3)</t>
-        </is>
-      </c>
+      <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, Quyết định VH-03</t>
+          <t>Bảng dữ liệu IN-32, Quyết định VH-03, Quyết định VH-10, Quyết định VH-11, Quyết định VH-12</t>
         </is>
       </c>
       <c r="Q6" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): design the vehicle model catalog
vehicle_models holds each model's specifications: weight, payload,
nominal battery capacity, an EV consumption curve by load and when the
manufacturer confirmed them; vehicles.make and model become
vehicle_model_id (VH-15). Electric figures only, no body type yet, and a
per-truck ADAS flag deferred (item 89).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -9576,7 +9576,7 @@
       </c>
       <c r="Q7" s="3" t="n"/>
     </row>
-    <row r="8" ht="40.5" customHeight="1">
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>SAF-04</t>
@@ -9647,7 +9647,7 @@
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-57, Bảng dữ liệu OUT-21, Điều kiện tiên quyết 7</t>
+          <t>Bảng dữ liệu IN-57, Bảng dữ liệu OUT-21, Điều kiện tiên quyết 7, deferred.md 89</t>
         </is>
       </c>
       <c r="Q8" s="3" t="n"/>
@@ -15088,7 +15088,7 @@
       </c>
       <c r="Q6" s="3" t="n"/>
     </row>
-    <row r="7" ht="40.5" customHeight="1">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>VEH-03</t>
@@ -15101,7 +15101,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Lưu thông số từng dòng xe (EVT-262/400/825): dung lượng pin, đường cong tiêu thụ theo tải và đường cơ sở xe diesel tương đương.</t>
+          <t>Lưu thông số từng dòng xe (EVT-262/400/825): dung lượng pin, đường cong tiêu thụ theo tải (chỉ số liệu xe điện).</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -15159,7 +15159,7 @@
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, Bảng dữ liệu IN-34, deferred.md 61, Quyết định VH-08</t>
+          <t>Bảng dữ liệu IN-32, Bảng dữ liệu IN-34, deferred.md 61, Quyết định VH-08, Quyết định VH-15</t>
         </is>
       </c>
       <c r="Q7" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): design the batteries table
One physical battery: serial, model, owner and installed truck each with
a since time under DM-22, one battery per truck, a decided status with a
reason, and views for its ownership and installation periods. A battery
the seller owns moves with the truck at a sale; vehicles loses
battery_capacity_kwh (VH-16). BAT-01 asks whether the BMS reports the
pack serial.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -15465,7 +15465,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="67.5" customHeight="1">
+    <row r="5" ht="94.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>BAT-01</t>
@@ -15495,7 +15495,8 @@
         <is>
           <t>• Danh mục dòng pin: hóa học (LFP/CATL), dung lượng thiết kế, điện áp, cấu trúc
 • Từng pin: số serial, dòng pin, chủ sở hữu (có thể khác chủ xe), trạng thái kèm lý do
-• Mỗi xe một pin; lịch sử pin đã được lắp trên xe nào</t>
+• Mỗi xe một pin; lịch sử pin đã được lắp trên xe nào
+• Pin thuộc bên bán chuyển sang bên mua khi xe được bán</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -15534,10 +15535,14 @@
         </is>
       </c>
       <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>• BMS của xe có gửi số serial của pin qua T-Box không? Nếu có, việc thay pin không được ghi nhận có thể phát cảnh báo.</t>
+        </is>
+      </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-33, Quyết định VH-08, Quyết định VH-13, deferred.md 87, deferred.md 88</t>
+          <t>Bảng dữ liệu IN-33, Quyết định VH-08, Quyết định VH-13, Quyết định VH-16, deferred.md 87, deferred.md 88</t>
         </is>
       </c>
       <c r="Q5" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): design warranties and narrow the tenant column
organization_id stays only as an entity's own owner or as the owner at
the time a record was made; rows that belong to a parent read it through
the parent (DM-24, replaces DM-18). The warranties domain gets its table:
one warranty of exactly one truck, battery or T-Box through three foreign
keys, no organization_id, limits as end counter readings (VH-18).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -12323,7 +12323,7 @@
       <c r="O19" s="3" t="n"/>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>Quyết định ID-11, Quyết định DM-18</t>
+          <t>Quyết định ID-11, Quyết định DM-24</t>
         </is>
       </c>
       <c r="Q19" s="3" t="n"/>
@@ -15763,7 +15763,7 @@
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, Quyết định VH-09, Quyết định VH-14</t>
+          <t>Bảng dữ liệu IN-32, Quyết định VH-09, Quyết định VH-14, Quyết định VH-18</t>
         </is>
       </c>
       <c r="Q5" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): review the telematics table
The T-Box profile keeps change history and an installed_at under DM-22;
status becomes ACTIVE, MAINTENANCE, DECOMMISSIONED with a reason; the
pushed interval stays as a decision while config_pushed_at goes; the
firmware moves to a new telematic_state table filled from the device's
status topic (TX-08, supersedes TX-03). Deferred item 30 is closed:
telematics stays its own domain.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -15980,7 +15980,7 @@
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-19, Bảng dữ liệu IN-20, Bảng dữ liệu IN-21, PRD F-G1, Quyết định TX-07</t>
+          <t>Bảng dữ liệu IN-19, Bảng dữ liệu IN-20, Bảng dữ liệu IN-21, PRD F-G1, Quyết định TX-07, Quyết định TX-08</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -16060,7 +16060,7 @@
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-19, PRD F-G1, Quyết định TX-02, Quyết định TX-03</t>
+          <t>Bảng dữ liệu IN-19, PRD F-G1, Quyết định TX-02, Quyết định TX-08</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): keep every T-Box status report
telematic_status_reports stores each health report a T-Box sends about
itself, append-only, so trends in signal, power and storage can be seen;
it follows the device to its next owner (TX-10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -16150,7 +16150,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="67.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>DEV-04</t>
@@ -16178,7 +16178,8 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>• Cờ online và im lặng tính từ dữ liệu mới nhất
+          <t>• Lịch sử sức khỏe theo từng thiết bị (sóng, nguồn điện, bộ nhớ, SIM) để xem xu hướng
+• Cờ online và im lặng tính từ dữ liệu mới nhất
 • Trạng thái SIM/ICCID, data, nguồn, bộ nhớ và GNSS
 • Tỷ lệ thiết bị khỏe trên toàn mạng</t>
         </is>
@@ -16222,7 +16223,7 @@
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>PRD F-J1, Bảng dữ liệu IN-21, Bảng dữ liệu IN-22, Bảng dữ liệu OUT-55, deferred.md 50</t>
+          <t>PRD F-J1, Bảng dữ liệu IN-21, Bảng dữ liệu IN-22, Bảng dữ liệu OUT-55, deferred.md 50, Quyết định TX-10</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): review the drivers table
A driver profile belongs to one membership and reads its organization
through it; name and phone stay on users. The licence stays on the profile
(number no longer unique, class, expiry), each organization keeping its own
copy; status gets a reason and the table gets change history (DR-09).
Ending a membership retires the profile; check-in eligibility and which
profile a session uses are defined, and a driver from another organization
only gives a warning (DR-10). Drivers see a summary of their own sessions,
cannot export them, and data requests go to the truck's owner (DR-11).
Driving time across organizations is open question 8. VH-08 and VH-09 are
marked designed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -7717,7 +7717,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="67.5" customHeight="1">
+    <row r="5" ht="108" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>SUP-01</t>
@@ -7748,7 +7748,8 @@
           <t>• Tạo yêu cầu với ngữ cảnh xe tự động và ảnh
 • Vòng đời mở → đã tiếp nhận → đã xử lý → đóng
 • Hạn SLA chốt khi tạo
-• Khiếu nại và báo lỗi phần mềm là các loại yêu cầu</t>
+• Khiếu nại và báo lỗi phần mềm là các loại yêu cầu
+• Yêu cầu dữ liệu là một loại yêu cầu: dữ liệu lái xe của chủ xe chỉ được cung cấp khi chủ xe đồng ý bằng văn bản hoặc có yêu cầu của cơ quan có thẩm quyền, và được ghi nhật ký</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -7794,7 +7795,7 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>PRD F-I1, Bảng dữ liệu IN-51, Bảng dữ liệu OUT-61</t>
+          <t>PRD F-I1, Bảng dữ liệu IN-51, Bảng dữ liệu OUT-61, Quyết định DR-11</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -19063,7 +19064,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="81" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>DRV-01</t>
@@ -19135,7 +19136,7 @@
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>PRD F-E4, Bảng dữ liệu IN-37, Bảng dữ liệu OUT-34, Quyết định ID-13, Quyết định DR-03</t>
+          <t>PRD F-E4, Bảng dữ liệu IN-37, Bảng dữ liệu OUT-34, Quyết định ID-13, Quyết định DR-03, Quyết định DR-09, Quyết định DR-10</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -19144,7 +19145,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="189" customHeight="1">
+    <row r="6" ht="229.5" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>DRV-02</t>
@@ -19177,7 +19178,7 @@
 • Mỗi xe một người cầm lái; phiên kết thúc khi trả xe, khi tài xế khác nhận xe, khi tài xế nhận xe khác, hoặc khi xe không di chuyển quá thời gian tự kết thúc của tổ chức (mặc định 2 giờ)
 • Cảnh báo lên portal khi xe chạy mà không ai nhận xe
 • Cảnh báo dành cho tài xế gửi tới tài xế đang nhận xe và portal
-• Lịch sử theo tài xế và theo xe</t>
+• Lịch sử đầy đủ theo tài xế và theo xe trên portal; tài xế chỉ xem bản tóm tắt các phiên của mình trên ứng dụng (không có lộ trình hay địa điểm, không xuất dữ liệu)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -19219,7 +19220,7 @@
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-07, Quyết định DR-08, Quyết định NT-07, Quyết định ID-45</t>
+          <t>PRD F-E4, Bảng dữ liệu IN-55, Bảng dữ liệu OUT-34, Quyết định DR-07, Quyết định DR-08, Quyết định DR-10, Quyết định DR-11, Quyết định NT-07, Quyết định ID-45</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
@@ -19388,7 +19389,7 @@
       </c>
       <c r="Q8" s="3" t="n"/>
     </row>
-    <row r="9" ht="40.5" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>DRV-05</t>
@@ -19457,7 +19458,11 @@
         </is>
       </c>
       <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>• Thời gian lái qua nhiều tổ chức: ai được xem tổng thời gian lái khi tài xế lái xe của nhiều tổ chức (câu hỏi mở 8, cố vấn pháp lý).</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Bảng dữ liệu IN-59, Bảng dữ liệu OUT-19</t>
@@ -19465,7 +19470,7 @@
       </c>
       <c r="Q9" s="3" t="n"/>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>DRV-06</t>
@@ -19533,7 +19538,11 @@
         </is>
       </c>
       <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>• Thời gian lái qua nhiều tổ chức: ai được xem tổng thời gian lái khi tài xế lái xe của nhiều tổ chức (câu hỏi mở 8, cố vấn pháp lý).</t>
+        </is>
+      </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Bảng dữ liệu OUT-39</t>

</xml_diff>

<commit_message>
docs(domain-model): defer charging credentials
Every charge at launch starts with a QR scan, including guest trucks, so no
charging credential is stored and the table leaves the design (CO-13). The
shape worked out for RFID cards and VIN Autocharge is kept in deferred.md
item 90 for when CHG-08 starts. CHG-07 asks whether the app takes a guest
truck's plate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -4910,7 +4910,11 @@
         </is>
       </c>
       <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>• Xe khách vãng lai (chưa đăng ký với chúng ta) không có hồ sơ xe: ứng dụng có hỏi biển số khi bắt đầu sạc bằng QR không?</t>
+        </is>
+      </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
           <t>deferred.md 62, Quyết định CO-12, Bảng dữ liệu IN-27</t>
@@ -4993,7 +4997,7 @@
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>Quyết định CO-12, Quyết định CO-06</t>
+          <t>Quyết định CO-12, Quyết định CO-06, Quyết định CO-13, deferred.md 90</t>
         </is>
       </c>
       <c r="Q12" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): split charging locations from chargers
Terms follow the industry (CS-09): a location is the place drivers go,
a charging station is one charger (one OCPP connection); the app and docs
show the Vietnamese words. Locations are owned by organizations, public or
private, with a per-location allow-list of other organizations
(charging_location_access, CS-10). A location has one address line, no
opening hours (always open, INACTIVE when closed) and sends charger alerts
to its owner's operations staff; a charger keeps only its profile, and what
it reports moves to charging_station_state (CS-11). The QR is shown on the
charger's screen and the driver starts and stops there (CO-14). Sites and
power groups are deferred (deferred.md 91).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -1095,7 +1095,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="27" customHeight="1">
+    <row r="12" ht="67.5" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>10</v>
       </c>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Trạm và trụ sạc, trạng thái realtime qua OCPP, sự cố, bản đồ trạm, hàng đợi, đặt chỗ và phân tải.</t>
+          <t>Trạm và trụ sạc, trạng thái realtime qua OCPP, sự cố, bản đồ trạm, hàng đợi, đặt chỗ và phân tải. Trong danh mục này "trạm" là nơi tài xế tới (bảng charging_locations) và "trụ" là một trụ sạc OCPP (bảng charging_stations), theo CS-09.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -2925,10 +2925,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="229.5" customHeight="1">
+    <row r="2" ht="526.5" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Trạm và trụ sạc, trạng thái realtime qua OCPP, sự cố, bản đồ trạm, hàng đợi, đặt chỗ và phân tải.</t>
+          <t>Trạm và trụ sạc, trạng thái realtime qua OCPP, sự cố, bản đồ trạm, hàng đợi, đặt chỗ và phân tải. Trong danh mục này "trạm" là nơi tài xế tới (bảng charging_locations) và "trụ" là một trụ sạc OCPP (bảng charging_stations), theo CS-09.</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="67.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>STN-01</t>
@@ -3055,7 +3055,7 @@
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>• Tạo, sửa, tìm kiếm và ngừng hoạt động trạm
-• Đơn vị quản lý và đầu mối sự cố của từng trạm
+• Tổ chức sở hữu của từng trạm; cảnh báo trụ sạc gửi tới nhân viên vận hành của tổ chức đó; trạm mở 24/7, trạm tạm đóng được đánh dấu ngừng hoạt động kèm lý do
 • Xem mọi trạm trên bản đồ</t>
         </is>
       </c>
@@ -3094,7 +3094,7 @@
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>PRD F-C1, Bảng dữ liệu IN-25</t>
+          <t>PRD F-C1, Bảng dữ liệu IN-25, Quyết định CS-09, Quyết định CS-10, Quyết định CS-11</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -3658,7 +3658,7 @@
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>PRD F-C7, Bảng dữ liệu IN-28, Bảng dữ liệu OUT-53, NF-20</t>
+          <t>PRD F-C7, Bảng dữ liệu IN-28, Bảng dữ liệu OUT-53, NF-20, deferred.md 91</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu OUT-10</t>
+          <t>Bảng dữ liệu OUT-10, Quyết định CS-10</t>
         </is>
       </c>
       <c r="Q16" s="3" t="n"/>
@@ -4363,7 +4363,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="81" customHeight="1">
+    <row r="5" ht="121.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CHG-01</t>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Tài xế quét mã QR trên trụ, hệ thống bắt đầu sạc từ xa, và app hiển thị tiến trình sạc tới khi dừng.</t>
+          <t>Tài xế quét mã QR trên màn hình trụ; ứng dụng xác thực và kiểm tra ví, tài xế bắt đầu và dừng sạc trên trụ, và ứng dụng hiển thị tiến trình.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4391,10 +4391,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>• Quét mã QR của súng sạc và xác nhận
+          <t>• Quét mã QR trên màn hình trụ sạc; ứng dụng xác thực tài xế và kiểm tra ví
+• Tài xế chọn súng và bắt đầu sạc trên màn hình trụ
 • Ghi nhận ai bắt đầu sạc và tổ chức nào trả tiền
 • Tiến trình realtime: kWh, % pin, công suất, chi phí tạm tính
-• Dừng từ app hoặc tại trụ
+• Dừng trên màn hình trụ (hoặc do xe tự dừng); ứng dụng không gửi lệnh
 • Giữ phiên và tính tiền sau nếu sóng yếu</t>
         </is>
       </c>
@@ -4434,10 +4435,14 @@
         </is>
       </c>
       <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>• Nhà cung cấp cần xác nhận: nội dung mã QR, chọn súng trên màn hình sau khi xác thực từ xa, AuthorizeRemoteTxRequests (câu hỏi mở 4).</t>
+        </is>
+      </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>PRD F-H1, Quyết định CO-12</t>
+          <t>PRD F-H1, Quyết định CO-12, Quyết định CO-13, Quyết định CO-14</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): review the charging topology tables
Locations get a required map point named coordinates and a duplicate-name
warning (CS-12). Location access gets an optional end date and a
revoke_reason, the naming rule for open/close tables without a status
(CS-13, DM-28). Chargers get a registered serial number (CS-14) and may
carry a warranty limited by energy and sessions (VH-19); their state keeps
latest values only and serves both protocols (CS-15). EVSEs get a status
and a public eMI3 ID (CS-16). Connectors get their standard and ratings,
closing deferred item 80, and their live status moves to a state table
(CS-17). Reservations leave the design (deferred.md 92).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -3103,7 +3103,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40.5" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>STN-02</t>
@@ -3174,7 +3174,7 @@
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Quyết định CS-02, Quyết định CS-03, deferred.md 80</t>
+          <t>Quyết định CS-02, Quyết định CS-03, deferred.md 80, Quyết định CS-16, Quyết định CS-17</t>
         </is>
       </c>
       <c r="Q6" s="3" t="n"/>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>PRD F-C4, Bảng dữ liệu IN-54</t>
+          <t>PRD F-C4, Bảng dữ liệu IN-54, deferred.md 92</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -15701,7 +15701,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="67.5" customHeight="1">
+    <row r="5" ht="94.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>WAR-01</t>
@@ -15714,7 +15714,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Lưu mọi bảo hành của xe, pin và thiết bị trên xe: thời hạn, các giới hạn như quãng đường hay số chu kỳ sạc, và trạng thái, kèm lý do khi bảo hành bị hủy.</t>
+          <t>Lưu mọi bảo hành của xe, pin, thiết bị trên xe và của trụ sạc: thời hạn, các giới hạn như quãng đường, số chu kỳ sạc, điện năng đã cấp hay số phiên sạc, và trạng thái, kèm lý do khi bảo hành bị hủy.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -15731,7 +15731,8 @@
         <is>
           <t>• Bảo hành theo từng xe, pin và thiết bị, đặt riêng cho từng xe, mỗi bảo hành có thời hạn và giới hạn riêng
 • Hết hạn được tính từ ngày và bộ đếm của xe hoặc pin; hủy bảo hành kèm lý do và lịch sử
-• Bảo hành của pin đi theo pin sang xe khác</t>
+• Bảo hành của pin đi theo pin sang xe khác
+• Bảo hành trụ sạc giới hạn theo điện năng đã cấp (kWh) và số phiên sạc, nhận diện theo số serial đã đăng ký</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -15773,7 +15774,7 @@
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-32, Quyết định VH-09, Quyết định VH-14, Quyết định VH-18</t>
+          <t>Bảng dữ liệu IN-32, Quyết định VH-09, Quyết định VH-14, Quyết định VH-18, Quyết định VH-19, Quyết định CS-14</t>
         </is>
       </c>
       <c r="Q5" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): design wallets, wallet transactions and payments
Launch with a personal prepaid wallet per user, topped up through payments
and debited per session bill; a minimum balance is checked at the scan and
an end-of-session overrun may go negative (BL-12 to BL-14). Payments hold
only real money through a gateway; the later company methods need no table
change. The wallet's legal boundaries are open question 11, and D5 is
answered for launch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -6248,7 +6248,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="40.5" customHeight="1">
+    <row r="11" ht="81" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>PAY-07</t>
@@ -6319,7 +6319,8 @@
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>• Quy tắc tiền cọc: cọc 300 nghìn, rút thì xử lý thế nào? (ghi chú bảng dữ liệu)</t>
+          <t>• Quy tắc tiền cọc: cọc 300 nghìn, rút thì xử lý thế nào? (ghi chú bảng dữ liệu)
+• Giới hạn pháp lý của số dư trả trước: chuyển, rút, hoàn tiền, cách gọi tên khi giới thiệu (câu hỏi mở 11 trong nhật ký quyết định).</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -6333,7 +6334,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="40.5" customHeight="1">
+    <row r="12" ht="67.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>PAY-08</t>
@@ -6403,7 +6404,7 @@
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>• Khi tài xế của đội xe đi sạc, ai trả tiền: tài xế hay doanh nghiệp? (quyết định mở D5)</t>
+          <t>• Thanh toán doanh nghiệp đến sau khi ra mắt: khi ra mắt mỗi người trả bằng ví của chính mình (BL-13); phương thức doanh nghiệp nào làm trước (ví tổ chức, hóa đơn tháng) vẫn cần chọn.</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): design trips as planned jobs and their execution
A fleet manager may plan a trip (A to B, planned times, driver, truck); the
driver checks in by QR, then presses Start and Finish, and the system
records the truck's T-Box position, odometer and battery % at both ends.
Trips move to the drivers domain; MON-11 is updated (DR-12).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -17529,7 +17529,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="54" customHeight="1">
+    <row r="15" ht="121.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>MON-11</t>
@@ -17542,7 +17542,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Chia luồng dữ liệu thành các chuyến (bắt đầu, điểm dừng, kết thúc) kèm quãng đường, năng lượng và thời gian từng chuyến; mỗi chuyến có mã để sau này gắn với đơn hàng.</t>
+          <t>Chuyến do quản lý đội xe lập kế hoạch (từ A tới B, giờ dự kiến, tài xế, xe) và được tài xế thực hiện bằng nút Bắt đầu và Kết thúc trên ứng dụng, kèm quãng đường, năng lượng và thời gian từng chuyến; mỗi chuyến có mã để sau này gắn với đơn hàng.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -17557,7 +17557,9 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>• Quy tắc xác định chuyến thống nhất với vận hành
+          <t>• Lập kế hoạch chuyến: từ A tới B, giờ đi và giờ đến dự kiến, tài xế và xe (không bắt buộc với tài xế tự chạy)
+• Tài xế bấm Bắt đầu và Kết thúc sau khi nhận xe; ghi vị trí T-Box, số km và phần trăm pin ở hai đầu
+• Nhắc khi xe chạy mà chưa bắt đầu chuyến; chuyến đang mở tự đóng khi phiên lái kết thúc
 • Km, kWh, kWh/km và chi phí theo chuyến
 • Lịch sử chuyến và chi phí trên app tài xế</t>
         </is>
@@ -17594,18 +17596,14 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>MON-09</t>
+          <t>MON-09, DRV-02</t>
         </is>
       </c>
       <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="inlineStr">
-        <is>
-          <t>• Thế nào là một chuyến? (bộ phận vận hành định nghĩa)</t>
-        </is>
-      </c>
+      <c r="O15" s="3" t="n"/>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-14, Bảng dữ liệu OUT-17, Bảng dữ liệu IN-40, deferred.md 46</t>
+          <t>Bảng dữ liệu IN-14, Bảng dữ liệu OUT-17, Bảng dữ liệu IN-40, deferred.md 46, Quyết định DR-12</t>
         </is>
       </c>
       <c r="Q15" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(domain-model): add notification recipients, defer the SMS channel
One row per alert and person with seen and read times (NT-10). Channels at
launch are the inbox, push and e-mail; the SMS channel moves to P1.1
(NT-11, deferred.md 96).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -1347,10 +1347,10 @@
         <v>8</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
@@ -1721,10 +1721,10 @@
         <v>178</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>9</v>
@@ -7123,7 +7123,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40.5" customHeight="1">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>NTF-03</t>
@@ -7162,7 +7162,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>P1.0</t>
+          <t>P1.1</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -7194,7 +7194,7 @@
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>PRD F-F3, Bảng dữ liệu IN-47, Quyết định BL-05</t>
+          <t>PRD F-F3, Bảng dữ liệu IN-47, Quyết định BL-05, Quyết định NT-11, deferred.md 96</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(domain-model): add organization notification settings, close notifications
An organization switches push and e-mail per kind of alert, storing only
exceptions to the defaults; the deliveries table is deferred with SMS and
NTF-07 moves to P1.1 (NT-12). This closes the notifications review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -1347,10 +1347,10 @@
         <v>8</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
@@ -1721,10 +1721,10 @@
         <v>178</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>9</v>
@@ -7470,7 +7470,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>P1.0</t>
+          <t>P1.1</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -7502,7 +7502,7 @@
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Bảng dữ liệu IN-47</t>
+          <t>Bảng dữ liệu IN-47, Quyết định NT-12</t>
         </is>
       </c>
       <c r="Q11" s="3" t="n"/>

</xml_diff>

<commit_message>
feat(charging-sessions): start charging by QR scan with remote start (WP8)
POST /charging-sessions/scan checks the charger, location, gun, wallet
minimum and creates the PENDING session, queues REMOTE_START for the
gateway and returns the token; stop, receipt, history, the pending-session
sweep and Authorize against issued tokens only (CE-20..CE-24).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -4363,7 +4363,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="121.5" customHeight="1">
+    <row r="5" ht="135" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CHG-01</t>
@@ -4395,7 +4395,7 @@
 • Tài xế chọn súng và bắt đầu sạc trên màn hình trụ
 • Ghi nhận ai bắt đầu sạc và tổ chức nào trả tiền
 • Tiến trình realtime: kWh, % pin, công suất, chi phí tạm tính
-• Dừng trên màn hình trụ (hoặc do xe tự dừng); ứng dụng không gửi lệnh
+• Dừng trên màn hình trụ (hoặc do xe tự dừng); ứng dụng cũng có thể gửi lệnh dừng từ xa cho người đã bắt đầu sạc
 • Giữ phiên và tính tiền sau nếu sóng yếu</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs: sync the feature catalog and docs with the finished refactor run
Backend status of the built features is now in the catalog (done or
doing), with related tables and open questions; architecture.md, the
domain boundary and dev-environment rules match the code; the plan lists
what was skipped and the debugging-phase next steps.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01URvQGCMdGQH5axXbsyq4p6
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -636,7 +636,7 @@
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>0/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -690,7 +690,7 @@
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -744,7 +744,7 @@
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -798,7 +798,7 @@
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>0/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>0/18</t>
+          <t>3/18</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1022,7 +1022,7 @@
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>0/7</t>
+          <t>3/7</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1076,7 +1076,7 @@
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>0/8</t>
+          <t>4/8</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>0/15</t>
+          <t>6/15</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1190,7 +1190,7 @@
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>0/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1300,7 +1300,7 @@
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>0/13</t>
+          <t>4/13</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1356,7 +1356,7 @@
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>0/8</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>0/176</t>
+          <t>57/176</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -2312,7 +2312,11 @@
           <t>ACC-01</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>fleets</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -2374,7 +2378,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -2392,7 +2396,11 @@
           <t>FLT-01, VEH-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>fleet_vehicle_memberships</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -2405,7 +2413,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40.5" customHeight="1">
+    <row r="7" ht="94.5" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>FLT-03</t>
@@ -2454,7 +2462,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -2472,8 +2480,16 @@
           <t>FLT-01, ACC-13</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>fleet_user_assignments</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>• Giới hạn đội xe đã áp dụng cho đội xe, dữ liệu xe, danh sách xe, phiên lái, chuyến đi và người nhận cảnh báo; chưa áp dụng cho danh sách thông báo của tổ chức, ca hỗ trợ, phiên sạc, hóa đơn, pin, bảo hành và các API chi tiết theo ID (xem Known issues trong kế hoạch refactor).</t>
+        </is>
+      </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Quyết định FL-03</t>
@@ -2531,7 +2547,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -2549,7 +2565,11 @@
           <t>FLT-02, MON-02, MON-09</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>fleets, fleet_vehicle_memberships, telemetry</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -2612,7 +2632,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -2630,7 +2650,11 @@
           <t>FLT-02, MON-01, NTF-01</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>geofences</t>
+        </is>
+      </c>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -3076,7 +3100,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3090,7 +3114,11 @@
         </is>
       </c>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>charging_locations, charging_stations, charging_evses, charging_connectors</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -3103,7 +3131,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="67.5" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>STN-02</t>
@@ -3152,7 +3180,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -3170,8 +3198,16 @@
           <t>STN-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>charging_stations, charging_evses, charging_connectors, charging_station_state</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>• Đặt trụ INACTIVE chỉ có hiệu lực ở lần bắt tay kết nối kế tiếp; trụ đang kết nối vẫn giữ kết nối đến khi nối lại (deferred.md 74).</t>
+        </is>
+      </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Quyết định CS-02, Quyết định CS-03, deferred.md 80, Quyết định CS-16, Quyết định CS-17</t>
@@ -3179,7 +3215,7 @@
       </c>
       <c r="Q6" s="3" t="n"/>
     </row>
-    <row r="7" ht="67.5" customHeight="1">
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>STN-03</t>
@@ -3230,7 +3266,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -3248,7 +3284,11 @@
           <t>STN-02</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>charging_stations, charging_station_state, charging_ocpp_messages, charging_station_configuration_captures, charging_station_configuration_entries</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
           <t>• Còn thiếu tài liệu từ nhà cung cấp: hướng dẫn tích hợp, bảng mã lỗi, thông tin công tơ, TLS/xác thực (câu hỏi mở 4).
@@ -3316,7 +3356,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -3334,8 +3374,16 @@
           <t>STN-03</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>charging_connector_state, charging_connectors</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>• Trạng thái được đánh dấu cũ khi trụ ngoại tuyến nhưng vẫn trả giá trị báo cáo cuối; quy tắc hết hạn thật là deferred.md 76.</t>
+        </is>
+      </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
           <t>PRD F-C2, Bảng dữ liệu IN-26, Bảng dữ liệu OUT-48, NF-02, deferred.md 76</t>
@@ -3802,7 +3850,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -3820,7 +3868,11 @@
           <t>STN-03</t>
         </is>
       </c>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>charging_station_commands</t>
+        </is>
+      </c>
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -3954,7 +4006,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -3972,7 +4024,11 @@
           <t>STN-01, PAY-09</t>
         </is>
       </c>
-      <c r="N16" s="3" t="n"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>charging_locations, charging_location_access</t>
+        </is>
+      </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
           <t>• Trụ riêng (của mỏ, không công cộng) tính tiền thế nào? Bảng dữ liệu ghi 'phương án riêng'.</t>
@@ -4416,7 +4472,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -4434,7 +4490,11 @@
           <t>STN-10, CHG-02, ACC-04</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions, charging_station_commands</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
           <t>• Nhà cung cấp cần xác nhận: nội dung mã QR, chọn súng trên màn hình sau khi xác thực từ xa, AuthorizeRemoteTxRequests (câu hỏi mở 4).</t>
@@ -4502,7 +4562,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -4520,7 +4580,11 @@
           <t>STN-03</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions, charging_session_measurements</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -4533,7 +4597,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="27" customHeight="1">
+    <row r="7" ht="40.5" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>CHG-03</t>
@@ -4582,7 +4646,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -4600,7 +4664,11 @@
           <t>CHG-02, PAY-10</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions, charging_session_bills</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -4658,7 +4726,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -4676,7 +4744,11 @@
           <t>CHG-02, CHG-07</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -4689,7 +4761,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="27" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>CHG-05</t>
@@ -4738,7 +4810,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -4756,8 +4828,16 @@
           <t>CHG-07</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions, charging_session_measurements</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có điện năng theo phiên và theo trụ; chưa có tổng theo tổ chức trong kỳ, và chủ trụ chỉ thấy phiên do tổ chức mình trả tiền.</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>PRD F-C6, Bảng dữ liệu OUT-51, deferred.md 62</t>
@@ -4896,7 +4976,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4914,7 +4994,11 @@
           <t>CHG-01, DRV-02</t>
         </is>
       </c>
-      <c r="N11" s="3" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>charging_sessions, driving_sessions</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>• Xe khách vãng lai (chưa đăng ký với chúng ta) không có hồ sơ xe: ứng dụng có hỏi biển số khi bắt đầu sạc bằng QR không?</t>
@@ -6167,7 +6251,7 @@
       </c>
       <c r="Q9" s="3" t="n"/>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="67.5" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>PAY-06</t>
@@ -6217,7 +6301,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -6235,8 +6319,16 @@
           <t>CHG-01, CHG-03</t>
         </is>
       </c>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>payments, wallets, charging_session_bills</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>• Cấu trúc mã VietQR theo chuẩn NAPAS nhưng chưa được quét thử bằng app ngân hàng thật; cần kiểm chứng với tài khoản thật đầu tiên. Thông báo ngân hàng đang dùng nhà cung cấp giả.</t>
+        </is>
+      </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>PRD F-H1, Bảng dữ liệu IN-45, NF-05</t>
@@ -6298,7 +6390,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -6316,7 +6408,11 @@
           <t>PAY-06</t>
         </is>
       </c>
-      <c r="N11" s="3" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>wallets, wallet_transactions, payments</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>• Quy tắc tiền cọc: cọc 300 nghìn, rút thì xử lý thế nào? (ghi chú bảng dữ liệu)
@@ -6468,7 +6564,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -6486,7 +6582,11 @@
           <t>STN-01, STN-13</t>
         </is>
       </c>
-      <c r="N13" s="3" t="n"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>tariffs, tariff_versions</t>
+        </is>
+      </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
           <t>• Ai sở hữu biểu giá (G3 Energy hay G3 Network), và chênh lệch giá cao điểm/thấp điểm bao nhiêu?</t>
@@ -6503,7 +6603,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
+    <row r="14" ht="40.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>PAY-10</t>
@@ -6552,7 +6652,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -6570,7 +6670,11 @@
           <t>PAY-09, CHG-02</t>
         </is>
       </c>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>charging_session_bills, tariff_versions</t>
+        </is>
+      </c>
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -7016,7 +7120,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -7030,7 +7134,11 @@
         </is>
       </c>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>notifications, notification_recipients</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -7043,7 +7151,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40.5" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>NTF-02</t>
@@ -7092,7 +7200,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -7110,8 +7218,16 @@
           <t>NTF-01, ACC-16, NTF-06</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>notification_recipients, user_sessions</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>• Thông báo đẩy đi qua nhà cung cấp giả và được gửi trong giao dịch của bên tạo; nhà cung cấp thật cần outbox gửi sau khi commit (deferred.md 100).</t>
+        </is>
+      </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
           <t>PRD F-F3, Quyết định ID-19, deferred.md 41</t>
@@ -7252,7 +7368,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -7270,8 +7386,16 @@
           <t>NTF-06</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>notification_recipients, notifications</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>• E-mail đi qua nhà cung cấp giả và được gửi trong giao dịch của bên tạo (deferred.md 100).</t>
+        </is>
+      </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
           <t>Quyết định NT-03</t>
@@ -7328,7 +7452,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -7346,7 +7470,11 @@
           <t>NTF-06</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>organization_notification_settings</t>
+        </is>
+      </c>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -7404,7 +7532,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -7422,7 +7550,11 @@
           <t>ACC-14, ACC-15</t>
         </is>
       </c>
-      <c r="N10" s="3" t="n"/>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>notifications, notification_recipients</t>
+        </is>
+      </c>
       <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="inlineStr">
         <is>
@@ -11220,7 +11352,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -11234,7 +11366,11 @@
         </is>
       </c>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>organizations, organization_settings</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -11296,7 +11432,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -11314,7 +11450,11 @@
           <t>ACC-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>organizations, users</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -11373,7 +11513,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -11387,7 +11527,11 @@
         </is>
       </c>
       <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>users, user_state, user_credentials</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -11454,7 +11598,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -11472,7 +11616,11 @@
           <t>ACC-03</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>user_credentials, user_sessions, user_state</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -11531,7 +11679,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -11549,7 +11697,11 @@
           <t>ACC-03, NTF-03</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>one_time_codes</t>
+        </is>
+      </c>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -11609,7 +11761,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -11627,8 +11779,16 @@
           <t>ACC-05</t>
         </is>
       </c>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>one_time_codes, user_credentials, users</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>• Chưa có bước xác minh thêm khi đặt lại mật khẩu tài khoản lâu không hoạt động (SĐT bị cấp lại) và giới hạn tần suất theo thiết bị (deferred.md 99).</t>
+        </is>
+      </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Quyết định ID-16, Rà soát thiết kế 2026-10-03</t>
@@ -11687,7 +11847,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -11705,7 +11865,11 @@
           <t>ACC-01, ACC-05, ACC-17, PAY-02</t>
         </is>
       </c>
-      <c r="N11" s="3" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>users, organizations, memberships, user_credentials, one_time_codes</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="inlineStr">
         <is>
@@ -11765,7 +11929,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -11783,7 +11947,11 @@
           <t>ACC-01, ACC-09, PAY-03</t>
         </is>
       </c>
-      <c r="N12" s="3" t="n"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>organizations, users, memberships, one_time_codes</t>
+        </is>
+      </c>
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="inlineStr">
         <is>
@@ -11842,7 +12010,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -11860,7 +12028,11 @@
           <t>ACC-05, ACC-12, ACC-13</t>
         </is>
       </c>
-      <c r="N13" s="3" t="n"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>memberships, users, one_time_codes, user_role_assignments</t>
+        </is>
+      </c>
       <c r="O13" s="3" t="n"/>
       <c r="P13" s="3" t="inlineStr">
         <is>
@@ -11918,7 +12090,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -11936,7 +12108,11 @@
           <t>ACC-09, DRV-01</t>
         </is>
       </c>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>memberships, drivers, one_time_codes, users</t>
+        </is>
+      </c>
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -12071,7 +12247,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -12089,7 +12265,11 @@
           <t>ACC-01, ACC-03</t>
         </is>
       </c>
-      <c r="N16" s="3" t="n"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>memberships</t>
+        </is>
+      </c>
       <c r="O16" s="3" t="n"/>
       <c r="P16" s="3" t="inlineStr">
         <is>
@@ -12148,7 +12328,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -12166,7 +12346,11 @@
           <t>ACC-12</t>
         </is>
       </c>
-      <c r="N17" s="3" t="n"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>user_role_assignments, memberships</t>
+        </is>
+      </c>
       <c r="O17" s="3" t="n"/>
       <c r="P17" s="3" t="inlineStr">
         <is>
@@ -12231,7 +12415,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -12249,7 +12433,11 @@
           <t>ACC-13, PAY-02</t>
         </is>
       </c>
-      <c r="N18" s="3" t="n"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>user_role_assignments, memberships</t>
+        </is>
+      </c>
       <c r="O18" s="3" t="n"/>
       <c r="P18" s="3" t="inlineStr">
         <is>
@@ -12312,7 +12500,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -12330,7 +12518,11 @@
           <t>ACC-12, FLT-03</t>
         </is>
       </c>
-      <c r="N19" s="3" t="n"/>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>memberships, organizations, fleet_user_assignments</t>
+        </is>
+      </c>
       <c r="O19" s="3" t="n"/>
       <c r="P19" s="3" t="inlineStr">
         <is>
@@ -12389,7 +12581,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -12407,7 +12599,11 @@
           <t>ACC-04</t>
         </is>
       </c>
-      <c r="N20" s="3" t="n"/>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>user_sessions</t>
+        </is>
+      </c>
       <c r="O20" s="3" t="n"/>
       <c r="P20" s="3" t="inlineStr">
         <is>
@@ -12468,7 +12664,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -12482,8 +12678,16 @@
         </is>
       </c>
       <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>user_consents, legal_documents</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>• Việc chấp nhận được ghi nhận, nhưng chưa có API nào từ chối sử dụng khi còn văn bản chưa chấp nhận; điểm áp dụng sẽ làm cùng bước cấp quyền (ID-44).</t>
+        </is>
+      </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
           <t>Bảng dữ liệu IN-37, NF-08, Quyết định ID-20, Quyết định ID-38, Quyết định ID-43</t>
@@ -12543,7 +12747,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -12557,7 +12761,11 @@
         </is>
       </c>
       <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>access_audit_logs</t>
+        </is>
+      </c>
       <c r="O22" s="3" t="n"/>
       <c r="P22" s="3" t="inlineStr">
         <is>
@@ -12701,7 +12909,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -12715,7 +12923,11 @@
         </is>
       </c>
       <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>users, user_role_assignments, access_audit_logs</t>
+        </is>
+      </c>
       <c r="O24" s="3" t="n"/>
       <c r="P24" s="3" t="inlineStr">
         <is>
@@ -14995,7 +15207,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -15009,7 +15221,11 @@
         </is>
       </c>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>vehicles, vehicle_models</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -15072,7 +15288,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -15090,7 +15306,11 @@
           <t>VEH-01, ACC-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>vehicles, organizations</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -15148,7 +15368,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -15166,7 +15386,11 @@
           <t>VEH-01</t>
         </is>
       </c>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>vehicle_models</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -15224,7 +15448,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -15242,7 +15466,11 @@
           <t>VEH-01, DEV-02</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>vehicles, telematics, telemetry</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -15527,7 +15755,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -15545,7 +15773,11 @@
           <t>VEH-01</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>batteries, battery_models</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
           <t>• BMS của xe có gửi số serial của pin qua T-Box không? Nếu có, việc thay pin không được ghi nhận có thể phát cảnh báo.</t>
@@ -15753,7 +15985,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -15771,7 +16003,11 @@
           <t>VEH-01, BAT-01</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>warranties</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -15974,7 +16210,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -15988,7 +16224,11 @@
         </is>
       </c>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>telematics</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -16050,7 +16290,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -16068,7 +16308,11 @@
           <t>DEV-01, VEH-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>telematics, vehicles</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -16131,7 +16375,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -16145,7 +16389,11 @@
         </is>
       </c>
       <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>telematics, telemetry, telematic_status_reports</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
           <t>• Đặc tả telematics của Tri-Ring (trường, tần suất, giao thức, quyền truy cập BMS) chưa được chốt; phương án dự phòng là gateway OBD/CAN bên thứ ba.</t>
@@ -16213,7 +16461,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -16231,7 +16479,11 @@
           <t>DEV-01, MON-01</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>telematics, telematic_status_reports, telemetry</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -16293,7 +16545,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -16311,7 +16563,11 @@
           <t>DEV-02, NTF-01</t>
         </is>
       </c>
-      <c r="N9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>telematics, telemetry, notifications</t>
+        </is>
+      </c>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -16763,7 +17019,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -16781,7 +17037,11 @@
           <t>DEV-03</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>telemetry, telematics</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -16843,7 +17103,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -16861,7 +17121,11 @@
           <t>MON-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>telemetry</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -17581,7 +17845,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -17599,7 +17863,11 @@
           <t>MON-09, DRV-02</t>
         </is>
       </c>
-      <c r="N15" s="3" t="n"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>trips, driving_sessions</t>
+        </is>
+      </c>
       <c r="O15" s="3" t="n"/>
       <c r="P15" s="3" t="inlineStr">
         <is>
@@ -19123,7 +19391,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -19141,7 +19409,11 @@
           <t>ACC-12</t>
         </is>
       </c>
-      <c r="N5" s="3" t="n"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>drivers, memberships</t>
+        </is>
+      </c>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -19207,7 +19479,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -19225,7 +19497,11 @@
           <t>DRV-01, VEH-01</t>
         </is>
       </c>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>driving_sessions, drivers</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -19367,7 +19643,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -19385,7 +19661,11 @@
           <t>DRV-02, SAF-03</t>
         </is>
       </c>
-      <c r="N8" s="3" t="n"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>driving_sessions, drivers</t>
+        </is>
+      </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
           <t>• Hai tài xế một xe: dùng một app hay hai app?</t>

</xml_diff>

<commit_message>
docs: charging test-day planner, runbook and decisions (CO-16, CO-17, CE-28, CE-29)
- New planner docs/planners/backend-charging-test-day.md: the external
  review's findings, decisions D1-D10, rehearsal evidence and the
  test-day runbook (server on the VM, A:9000 -> B:9000, phases 1-3).
- Decision log: CO-16 (naive time as UTC, transaction messages always
  confirmed; supersedes CO-10), CO-17 (schema check also skipped for
  Boot/Status/Start; supersedes CO-08), CE-28 (A-Z0-9 token), CE-29
  (staff force-close); deferred.md 101 (who force-closed, logged only).
- Feature catalog: CHG-02 gains the force-close capability; sources.
- architecture.md, dev-environment.md, README, scenario files, the
  e2e-sim and ocpp-reference skills, pointers in the 1.6J planner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -3297,7 +3297,7 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>PRD F-G2, Quyết định CO-01, Quyết định CO-02, Quyết định CO-05</t>
+          <t>PRD F-G2, Quyết định CO-01, Quyết định CO-02, Quyết định CO-05, Quyết định CO-16, Quyết định CO-17</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>PRD F-H1, Quyết định CO-12, Quyết định CO-13, Quyết định CO-14, Quyết định CE-10, Quyết định CE-11</t>
+          <t>PRD F-H1, Quyết định CO-12, Quyết định CO-13, Quyết định CO-14, Quyết định CE-10, Quyết định CE-11, Quyết định CE-28</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -4511,7 +4511,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="81" customHeight="1">
+    <row r="6" ht="108" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>CHG-02</t>
@@ -4542,7 +4542,8 @@
           <t>• Vòng đời phiên từ bản tin của trụ
 • Mọi chỉ số đo (điện năng, công suất, điện áp, dòng, % pin, nhiệt độ)
 • Không sửa được sau khi kết thúc
-• Xử lý gửi lại, trùng lặp và sai thứ tự</t>
+• Xử lý gửi lại, trùng lặp và sai thứ tự
+• Nhân viên đóng phiên mà trụ không bao giờ kết thúc (trụ khởi động lại hoặc mất điện giữa phiên)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -4588,7 +4589,7 @@
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>PRD F-B2, Bảng dữ liệu IN-27, NF-11, deferred.md 27, Quyết định CE-10, Quyết định CE-12, Quyết định CE-14, Quyết định CE-15</t>
+          <t>PRD F-B2, Bảng dữ liệu IN-27, NF-11, deferred.md 27, Quyết định CE-10, Quyết định CE-12, Quyết định CE-14, Quyết định CE-15, Quyết định CO-16, Quyết định CE-29, deferred.md 101</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: resolve deferred 74 (command channel built), supersede CO-05 by CO-18
- deferred.md 74 moves to deferred-resolved.md: the command channel and
  its eight commands were built on 2026-10-10 (CS-24) and the sessions
  side of a remote start in WP8. The remainder - Smart Charging,
  firmware/diagnostics, reservation, closing an open connection, several
  gateway processes - is the new item 102.
- CO-05 ("the only CSMS-initiated call is the post-boot GetConfiguration")
  was no longer true; CO-18 restates it with the command channel. Live
  references (DBML note and views, STN-03 sources, two docstrings,
  deferred 93) point to CO-18; history files keep CO-05.
- 1.6J planner: dated pointers on the coverage table (Authorize, the
  command row) and the out-of-scope table; the ocpp-reference skill's
  deferred list is current (#80 was resolved, #74 is now #102).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -3205,7 +3205,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>• Đặt trụ INACTIVE chỉ có hiệu lực ở lần bắt tay kết nối kế tiếp; trụ đang kết nối vẫn giữ kết nối đến khi nối lại (deferred.md 74).</t>
+          <t>• Đặt trụ INACTIVE chỉ có hiệu lực ở lần bắt tay kết nối kế tiếp; trụ đang kết nối vẫn giữ kết nối đến khi nối lại (deferred.md 102).</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>PRD F-G2, Quyết định CO-01, Quyết định CO-02, Quyết định CO-05, Quyết định CO-16, Quyết định CO-17</t>
+          <t>PRD F-G2, Quyết định CO-01, Quyết định CO-02, Quyết định CO-16, Quyết định CO-17, Quyết định CO-18</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -3800,7 +3800,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="40.5" customHeight="1">
+    <row r="14" ht="67.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>STN-10</t>
@@ -3876,7 +3876,7 @@
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Quyết định CO-12, deferred.md 74, Quyết định CS-20</t>
+          <t>Quyết định CO-12, deferred.md 74, Quyết định CS-20, Quyết định CS-24, Quyết định CO-18, deferred.md 102</t>
         </is>
       </c>
       <c r="Q14" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(catalog): backend status of features built under their old codes
MON-10, STN-14 and SUP-02 are done on the backend; MON-04..07, MON-14,
STN-06 and SUP-01 are partly built, each with a note on what is built and
what is missing. The 2026-10-10 sync had left them at todo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -912,7 +912,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>3/18</t>
+          <t>4/18</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>6/15</t>
+          <t>7/15</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1412,7 +1412,7 @@
       <c r="J17" s="3" t="n"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>0/7</t>
+          <t>1/7</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>57/176</t>
+          <t>60/176</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="Q9" s="3" t="n"/>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="81" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>STN-06</t>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -3541,7 +3541,11 @@
         </is>
       </c>
       <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có ở backend: tìm trạm gần theo bán kính, lọc đang trống, công suất tối thiểu, chuẩn đầu sạc, kèm số súng trống (F-D1). Chưa có: giá hiện tại trong từng kết quả (giá đang lấy riêng theo từng trụ từ phần thanh toán).</t>
+        </is>
+      </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>PRD F-D1, Bảng dữ liệu OUT-5</t>
@@ -4167,7 +4171,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -7912,7 +7916,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -7933,7 +7937,8 @@
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>• Ai trực CSKH 24/7 (nội bộ hay thuê ngoài), và cam kết được SLA nào?</t>
+          <t>• Ai trực CSKH 24/7 (nội bộ hay thuê ngoài), và cam kết được SLA nào?
+• Đã có ở backend: ticket kèm VIN, vị trí và mã lỗi do app gửi, kênh app/Zalo/hotline, vòng đời mở → đã tiếp nhận → đã xử lý → đóng, hạn SLA phản hồi chốt khi tạo (F-I1). Chưa có: ảnh, và các loại khiếu nại, báo lỗi phần mềm, yêu cầu dữ liệu.</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -7997,7 +8002,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -17224,7 +17229,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="67.5" customHeight="1">
+    <row r="8" ht="108" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>MON-04</t>
@@ -17274,7 +17279,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -17295,7 +17300,8 @@
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>• Ngưỡng 30/20/10% cần chốt sau khi phỏng vấn tài xế.</t>
+          <t>• Ngưỡng 30/20/10% cần chốt sau khi phỏng vấn tài xế.
+• Đã có ở backend: cảnh báo khi pin giảm qua ngưỡng 30/20/10%, kèm trạm trống gần nhất chốt tại thời điểm cảnh báo (F-A2). Chưa có: ngưỡng đang cố định trong mã (MON-17), và cảnh báo lặp lại mỗi lần pin giảm qua ngưỡng chứ chưa phải một lần mỗi chuyến.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -17360,7 +17366,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -17379,7 +17385,11 @@
         </is>
       </c>
       <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có ở backend: cảnh báo nhiệt độ cao (≥60 °C) và sụt áp đột ngột (F-A4). Chưa có: cảnh báo cell/module, mất cân bằng, cách điện, contactor và làm mát, và nhắc lại khi tình trạng còn kéo dài.</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>PRD F-A4, Bảng dữ liệu IN-7, Bảng dữ liệu IN-8, Bảng dữ liệu OUT-4, deferred.md 43, deferred.md 44</t>
@@ -17441,7 +17451,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -17460,7 +17470,11 @@
         </is>
       </c>
       <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có ở backend: mã lỗi từ thiết bị tạo cảnh báo bất thường kèm mã gốc (F-A4). Chưa có: dịch mã qua bảng mã lỗi (VEH-06, chờ bảng của nhà sản xuất), tín hiệu trạng thái thiết bị và bảng tổng hợp lỗi của đội xe.</t>
+        </is>
+      </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>PRD F-A4, Bảng dữ liệu IN-9, Bảng dữ liệu IN-10, Bảng dữ liệu IN-16, Bảng dữ liệu OUT-4, Bảng dữ liệu OUT-27, deferred.md 42, deferred.md 45</t>
@@ -17472,7 +17486,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="54" customHeight="1">
+    <row r="11" ht="67.5" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>MON-07</t>
@@ -17522,7 +17536,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -17541,7 +17555,11 @@
         </is>
       </c>
       <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có ở backend: xu hướng SOH và số chu kỳ theo ngày, cảnh báo SOH dưới ngưỡng cấu hình (F-A3). Chưa có: dung lượng khả dụng ước tính, và định nghĩa SOH, chu kỳ thống nhất với nhà sản xuất.</t>
+        </is>
+      </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
           <t>PRD F-A3, Bảng dữ liệu IN-4, Bảng dữ liệu IN-5, Điều kiện tiên quyết 1</t>
@@ -17763,7 +17781,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -18040,7 +18058,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="67.5" customHeight="1">
+    <row r="18" ht="81" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>MON-14</t>
@@ -18090,7 +18108,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -18109,7 +18127,11 @@
         </is>
       </c>
       <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>• Đã có ở backend: quãng đường, năng lượng và các chỉ số theo xe, chia theo ngày, tuần, tháng, xuất CSV (F-A6). Chưa có: chi phí đang tính theo một giá cố định mỗi kWh trong cấu hình, chưa theo biểu giá áp dụng (PAY-09).</t>
+        </is>
+      </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
           <t>PRD F-A6, Bảng dữ liệu OUT-17, deferred.md 60, deferred.md 64</t>

</xml_diff>

<commit_message>
docs: owner confirms FL-15 (rows with no truck); defer the production setup (106)
The hardening planner is done and moves to docs/planners/done/. Deferred
item 106 records the production deployment setup (VPS, TLS, secrets, real
providers, freezing the baseline migration), which the owner deferred.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -2413,7 +2413,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="108" customHeight="1">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>FLT-03</t>
@@ -2485,11 +2485,7 @@
           <t>fleet_user_assignments</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>• Dữ liệu không gắn xe (D5, FL-15, đang giả định): thông báo và ca hỗ trợ không gắn xe vẫn hiện với quản lý bị giới hạn đội; phiên sạc và hóa đơn không gắn xe (trừ của chính người đó), pin trong kho, thiết bị chưa lắp, bảo hành của chúng, bảo hành trụ sạc và chuyến đi không có xe bị ẩn. Chờ chủ dự án xác nhận.</t>
-        </is>
-      </c>
+      <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Quyết định FL-03, Quyết định FL-13, Quyết định FL-14, Quyết định FL-15, Quyết định FL-16</t>

</xml_diff>

<commit_message>
docs: ID-54 feature list of /auth/me and ACC-23 organization settings; D11 updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>4</v>
@@ -636,7 +636,7 @@
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>0/19</t>
+          <t>0/20</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -1718,10 +1718,10 @@
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>17</v>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>61/176</t>
+          <t>62/177</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>0/138</t>
+          <t>0/139</t>
         </is>
       </c>
     </row>
@@ -11172,7 +11172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13086,6 +13086,82 @@
         </is>
       </c>
       <c r="Q26" s="3" t="n"/>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>ACC-23</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Cài đặt tổ chức</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Cho quản trị viên của tổ chức chọn cách hệ thống hoạt động cho tổ chức mình: phiên lái xe không hoạt động tự kết thúc sau bao lâu, xe gửi dữ liệu bao lâu một lần.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Mỗi khách hàng tự chỉnh quy tắc theo cách vận hành xe của mình, không cần nhờ chúng tôi.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Quản trị tổ chức, Đồng quản trị (nội bộ), Quản trị trưởng (nội bộ)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>• Thời gian tự kết thúc phiên lái xe và chu kỳ gửi dữ liệu, trong giới hạn cho phép
+• Mỗi thay đổi cần lý do và được lưu trong lịch sử thay đổi</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Bắt buộc</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>P1.0</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Có trong mọi gói</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Không cần</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>organization_settings</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="n"/>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định ID-45</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
docs: web portal scaffold done; conventions, architecture, README and catalog in line
The scaffold planner is finished (Steps 1-8) and moves to planners/done/.
The portal rules record what the build settled (shell through InnerWrap,
guards, typed i18n keys, status labels in common, Form.Item extra for help
text, FilterField, Playwright targets and the Ubuntu 20.04 browser note);
architecture.md and README describe the portal as it exists; the catalog
marks ACC-04, ACC-14, VEH-01 and FLT-04 portal: doing; TT-28, TT-29, CV-24
and CV-25 are built; deferred items 108 (date-picker month names) and 109
(live map beyond 100 trucks).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/features/features.xlsx
+++ b/docs/product/features/features.xlsx
@@ -2553,7 +2553,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -15295,7 +15295,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="M5" s="3" t="n"/>

</xml_diff>